<commit_message>
updated final working hours
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta Laura.xlsx
+++ b/docs/Työajan seuranta Laura.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bb667e905e7871ab/Documents/Git/movieproject/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="8_{42E345A2-8A07-4841-BEA8-AE5A2DA5432A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97EE4E03-E1B0-481F-AD04-2F306DC729A7}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="8_{42E345A2-8A07-4841-BEA8-AE5A2DA5432A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AAF8A21-44F6-48A0-AB7F-78E6C3A1D897}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="71">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -239,6 +239,51 @@
   </si>
   <si>
     <t>1.25 h</t>
+  </si>
+  <si>
+    <t>7.10.</t>
+  </si>
+  <si>
+    <t>Projektin etenemisen tarkastelu ja tehtävien päivittäminen</t>
+  </si>
+  <si>
+    <t>1 h</t>
+  </si>
+  <si>
+    <t>11.10.</t>
+  </si>
+  <si>
+    <t>Projektin palautettavien materiaalien tarkistaminen
+Palaveria</t>
+  </si>
+  <si>
+    <t>12.10.</t>
+  </si>
+  <si>
+    <t>Loppuesityksen valmistelu
+Palaveria</t>
+  </si>
+  <si>
+    <t>1.50 h</t>
+  </si>
+  <si>
+    <t>13.10.</t>
+  </si>
+  <si>
+    <t>Sovellusdemon oman osuuden valmistelu</t>
+  </si>
+  <si>
+    <t>14.10.</t>
+  </si>
+  <si>
+    <t>Esityksen harjoittelemista
+Palaveria</t>
+  </si>
+  <si>
+    <t>15.10.</t>
+  </si>
+  <si>
+    <t>Loppuesityksen harjoittelu (kenraali)</t>
   </si>
 </sst>
 </file>
@@ -306,10 +351,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -609,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BD4D073-EB2D-44A2-86BF-660E3721AF80}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" customWidth="1"/>
@@ -879,6 +920,72 @@
       </c>
       <c r="C22" s="1" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -896,14 +1003,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009BAF6AFB37B6774A9122C6036818BC92" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c611cd0fe7e35dfe638a44e659100205">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44038759-07ae-40d4-bc3d-7c9fb0b3775b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36a43d4c38ea7f7b42b5de64d2c1c906" ns3:_="">
     <xsd:import namespace="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
@@ -1083,6 +1182,14 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
   <ds:schemaRefs>
@@ -1092,16 +1199,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1119,6 +1216,16 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{9f9ce49a-5101-4aa3-8c75-0d5935ad6525}" enabled="0" method="" siteId="{9f9ce49a-5101-4aa3-8c75-0d5935ad6525}" removed="1"/>

</xml_diff>